<commit_message>
Implement wave 1 scalability fix operating layer
</commit_message>
<xml_diff>
--- a/docs/ops/CEO_WEEKLY_SCORECARD.xlsx
+++ b/docs/ops/CEO_WEEKLY_SCORECARD.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deals" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clients" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Priorities" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operating Rules" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -431,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -507,6 +508,42 @@
       <c r="B6" t="inlineStr">
         <is>
           <t>Focus op revenue + proof en delivery stability; geen nieuwe grote projecten buiten deze command window.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Lead source of truth</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Verisight_CRM.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Delivery source of truth</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>/beheer en /campaigns/[id]</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Mirror rule</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Deals en Clients zijn weekmirrors; werk eerst het primaire systeem bij.</t>
         </is>
       </c>
     </row>
@@ -521,7 +558,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -621,32 +658,48 @@
       <c r="D5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Revenue proof</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Gekwalificeerde gesprekken deze week</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr"/>
-      <c r="D6" s="2" t="inlineStr"/>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Current frame</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Lead source of truth</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Verisight_CRM.xlsx</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Werk eerst de CRM-pipeline bij en spiegel daarna naar Deals.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Revenue proof</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Lopende proposals/offertes</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr"/>
-      <c r="D7" s="2" t="inlineStr"/>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Current frame</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Delivery source of truth</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>/beheer en /campaigns/[id]</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Werk eerst de app-deliverylaag bij en spiegel daarna naar Clients.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -656,7 +709,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Betaalde klanten of pilots in flight</t>
+          <t>Gekwalificeerde gesprekken deze week</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr"/>
@@ -670,7 +723,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Win rate rolling 30 dagen</t>
+          <t>Lopende proposals/offertes</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr"/>
@@ -684,7 +737,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Doorlooptijd gesprek naar voorstel</t>
+          <t>Betaalde klanten of pilots in flight</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr"/>
@@ -698,7 +751,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Nieuwe case-proof snippets deze week</t>
+          <t>Win rate rolling 30 dagen</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr"/>
@@ -712,7 +765,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Grootste bezwaar</t>
+          <t>Doorlooptijd gesprek naar voorstel</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr"/>
@@ -726,25 +779,21 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>ICP-kwaliteit</t>
+          <t>Nieuwe case-proof snippets deze week</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>sterk / gemengd / diffuus</t>
-        </is>
-      </c>
+      <c r="D13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Delivery stability</t>
+          <t>Revenue proof</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Actieve klanttrajecten</t>
+          <t>Grootste bezwaar</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr"/>
@@ -753,16 +802,20 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Delivery stability</t>
+          <t>Revenue proof</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Trajecten met hoog risico</t>
+          <t>ICP-kwaliteit</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr"/>
-      <c r="D15" s="2" t="inlineStr"/>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>sterk / gemengd / diffuus</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -772,7 +825,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Delivery defects deze week</t>
+          <t>Actieve klanttrajecten</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr"/>
@@ -786,7 +839,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Handmatige escalaties</t>
+          <t>Trajecten met hoog risico</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr"/>
@@ -800,7 +853,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Dagen akkoord naar live start</t>
+          <t>Delivery defects deze week</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr"/>
@@ -814,7 +867,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Dagen live start naar eerste managementwaarde</t>
+          <t>Handmatige escalaties</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr"/>
@@ -828,7 +881,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Trajecten met expliciete vervolgstap</t>
+          <t>Dagen akkoord naar live start</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr"/>
@@ -837,12 +890,12 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Cash and capacity</t>
+          <t>Delivery stability</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Verwachte omzet komende 30 dagen</t>
+          <t>Dagen live start naar eerste managementwaarde</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr"/>
@@ -851,12 +904,12 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Cash and capacity</t>
+          <t>Delivery stability</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Verwachte omzet komende 90 dagen</t>
+          <t>Trajecten met expliciete vervolgstap</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr"/>
@@ -870,7 +923,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Openstaande facturatie of cashrisico</t>
+          <t>Verwachte omzet komende 30 dagen</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr"/>
@@ -884,7 +937,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Founder-capaciteit komende 14 dagen</t>
+          <t>Verwachte omzet komende 90 dagen</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr"/>
@@ -898,11 +951,39 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Initiatieven buiten kernroute</t>
+          <t>Openstaande facturatie of cashrisico</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr"/>
       <c r="D25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Cash and capacity</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Founder-capaciteit komende 14 dagen</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr"/>
+      <c r="D26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Cash and capacity</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Initiatieven buiten kernroute</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr"/>
+      <c r="D27" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -915,7 +996,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -951,20 +1032,25 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Next action</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Due date</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Biggest objection</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -981,7 +1067,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:K1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1019,30 +1105,35 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Intake complete</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Import ready</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Activation ready</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Report delivered</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>First management use</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Next step</t>
         </is>
@@ -1090,8 +1181,6 @@
           <t>Top priority</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1099,8 +1188,6 @@
           <t>Top priority</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1108,8 +1195,6 @@
           <t>Top priority</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1117,8 +1202,6 @@
           <t>Explicitly not doing</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1126,8 +1209,6 @@
           <t>Explicitly not doing</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1135,8 +1216,6 @@
           <t>Explicitly not doing</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1144,8 +1223,6 @@
           <t>Decision log follow-up</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1153,8 +1230,104 @@
           <t>Decision log follow-up</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Primary system</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Weekly mirror</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Rule</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Leads</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Verisight_CRM.xlsx</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Deals</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Deals is alleen een weekmirror van de live CRM-pipeline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Delivery</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>/beheer en /campaigns/[id]</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Clients is alleen een weekmirror van de live deliverylaag.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Weekly Scorecard</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Gebruik alleen echte data of noteer nog niet gemeten.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add roadmap priorities and simplify weekly focus
</commit_message>
<xml_diff>
--- a/docs/ops/CEO_WEEKLY_SCORECARD.xlsx
+++ b/docs/ops/CEO_WEEKLY_SCORECARD.xlsx
@@ -8,11 +8,12 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Scorecard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deals" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clients" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Priorities" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operating Rules" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Focus" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Scorecard" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deals" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clients" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Priorities" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operating Rules" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -558,6 +559,185 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="68" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Prompt</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Week van</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr"/>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Kies alleen de week die nu loopt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Deze week telt vooral</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr"/>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Welke ene beweging maakt deze week succesvol?</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Belangrijkste commerciële push</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr"/>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Welk gesprek, voorstel of outbound-batch moet deze week echt bewegen?</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Belangrijkste delivery-risk</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Welk klanttraject vraagt nu de meeste aandacht?</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Topprioriteit 1</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr"/>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Hou het concreet en uitvoerbaar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Topprioriteit 2</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr"/>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Alleen invullen als je het deze week echt doet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Topprioriteit 3</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr"/>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Alleen invullen als je het deze week echt doet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Niet doen 1</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr"/>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Wat laat je deze week bewust liggen?</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Niet doen 2</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr"/>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Wat laat je deze week bewust liggen?</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Niet doen 3</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr"/>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Wat laat je deze week bewust liggen?</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Besluit deze week</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr"/>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Welk besluit moet expliciet in de decision log landen?</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -658,44 +838,44 @@
       <c r="D5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Current frame</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Lead source of truth</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Verisight_CRM.xlsx</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>Werk eerst de CRM-pipeline bij en spiegel daarna naar Deals.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Current frame</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Delivery source of truth</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>/beheer en /campaigns/[id]</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>Werk eerst de app-deliverylaag bij en spiegel daarna naar Clients.</t>
         </is>
@@ -990,7 +1170,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1003,10 +1183,11 @@
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="32" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="42" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="42" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1050,7 +1231,7 @@
           <t>Biggest objection</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -1061,7 +1242,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1074,12 +1255,13 @@
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="32" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="32" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1133,7 +1315,7 @@
           <t>First management use</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Next step</t>
         </is>
@@ -1144,7 +1326,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1181,6 +1363,8 @@
           <t>Top priority</t>
         </is>
       </c>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1188,6 +1372,8 @@
           <t>Top priority</t>
         </is>
       </c>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1195,6 +1381,8 @@
           <t>Top priority</t>
         </is>
       </c>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1202,6 +1390,8 @@
           <t>Explicitly not doing</t>
         </is>
       </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1209,6 +1399,8 @@
           <t>Explicitly not doing</t>
         </is>
       </c>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1216,6 +1408,8 @@
           <t>Explicitly not doing</t>
         </is>
       </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1223,6 +1417,8 @@
           <t>Decision log follow-up</t>
         </is>
       </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1230,13 +1426,15 @@
           <t>Decision log follow-up</t>
         </is>
       </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1244,24 +1442,30 @@
   </sheetPr>
   <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="72" customWidth="1" min="4" max="4"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Primary system</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Weekly mirror</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Rule</t>
         </is>

</xml_diff>